<commit_message>
feat: 补充2025年1-11月数据，数据范围扩展至2025-01-01 ~ 2026-07-06
新增2025年1月-11月共335天数据，数据总量达552天（19个月），
支持日/周/月三种粒度的DAU与社区首页UV趋势分析及功能渗透率。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/社区评论需求汇总.xlsx
+++ b/社区评论需求汇总.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="社区评论需求汇总" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'社区评论需求汇总'!$A$1:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'社区评论需求汇总'!$A$1:$M$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,22 +438,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,50 +529,58 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>9.4.0 (20251203)</t>
+          <t>7.23.0 (2024Q3)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>评论区发图</t>
+          <t>社区-话题</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>支持用户在评论中发布图片，包含图片上传、预览、删除功能；后端评论存储结构扩展支持图片字段；适配iOS/Android双端</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>2</v>
+          <t>社区话题功能：首页话题卡片、帖子来源标签、话题榜搜索、话题详情页（结构+内容+评论列表）、话题定制分享</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>张伟/李明</t>
+          <t>王战胜/臧宝亮</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>王芳</t>
+          <t>周颖</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-55968</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>需兼容已有评论展示；图片需接入审核</t>
+          <t>延期至7/26开始开发，因UI确认和搜索需求变更</t>
         </is>
       </c>
     </row>
@@ -582,39 +590,43 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>9.4.0 (20251203)</t>
+          <t>8.0.0 (2024Q3)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>社区帖子推荐优化</t>
+          <t>社区个人主页改版&amp;IM即时通信</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>优化社区首页Feed流推荐算法，增加基于用户兴趣的个性化推荐；新增'推荐'Tab页，合并原有'关注'和'发现'</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>3</v>
+          <t>社区个人主页改版(IP属地/创作数/热门帖子标签/帖子搜索/转评赞历史) + IM即时通信(用户鉴权/在线状态/拉黑/举报/@功能/草稿箱/长文发帖/回复盖楼)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>李明/张伟</t>
+          <t>王战胜/臧宝亮</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>王芳</t>
+          <t>周颖</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -622,10 +634,14 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-57198</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>涉及推荐策略调整，需A/B测试</t>
+          <t>v8.0.0重点需求，含IM SDK集成</t>
         </is>
       </c>
     </row>
@@ -635,48 +651,60 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>9.4.0 (20251203)</t>
+          <t>8.0.0 (2024Q3)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>帖子点赞动效优化</t>
+          <t>消息中心改版</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>优化帖子点赞按钮的交互动效，增加点赞动画、点赞数实时更新；大V点赞特殊标识</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>1</v>
+          <t>消息中心全面改版：财经资讯改版、交易提醒、热门事件、互动消息（社区/产品回复）、订阅更新、消息未读数</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>张伟</t>
+          <t>李克林/卢浩</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>王芳</t>
+          <t>胡金鑫</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-57562</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>含互动消息（社区、产品回复）</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -684,52 +712,48 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>9.6.0 (20260114)</t>
+          <t>8.0.0 (2024Q3)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>创作者中心V2</t>
+          <t>点击新闻和724评论头像进个人主页</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>创作者中心二期建设：新增数据看板（阅读量/互动量/粉丝增长趋势）、内容管理后台（批量编辑/定时发布）、收益提现模块</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>4</v>
-      </c>
+          <t>在新闻和724快讯的评论区域点击用户头像进入个人主页</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>李明/张伟</t>
+          <t>李克林/卢浩</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>刘洋</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>依赖社区数据中台V2接口</t>
-        </is>
-      </c>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-57198</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -737,47 +761,47 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>9.6.0 (20260114)</t>
+          <t>8.0.0 (2024Q3)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>帖子评论排序优化</t>
+          <t>社区公约</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>评论支持按热度/时间排序切换；热评默认置顶；评论楼中楼展开优化</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>2</v>
-      </c>
+          <t>社区公约功能展示</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>张伟</t>
+          <t>李克林/卢浩</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>刘洋</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-57198</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -786,52 +810,48 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>9.6.0 (20260114)</t>
+          <t>8.1.0 (2024Q4)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Feed流性能优化</t>
+          <t>社区个人主页分享海报</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>优化社区首页Feed流滑动性能，实现虚拟列表、图片懒加载、预加载策略</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>2</v>
-      </c>
+          <t>社区个人主页支持生成分享海报</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>李明/张伟/王强</t>
+          <t>杨怀展/卢浩</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>刘洋</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Harmony端需单独适配</t>
-        </is>
-      </c>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58643</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -839,50 +859,58 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>9.8.0 (20260318)</t>
+          <t>8.1.1 (2024Q4)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>社区搜索V3</t>
+          <t>社区消息类型push</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>社区搜索三期：支持帖子全文搜索、搜索联想词、搜索结果按分类筛选（帖子/用户/话题）、热门搜索榜</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>3</v>
+          <t>社区消息类型推送通知</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>李明/张伟</t>
+          <t>杨怀展/卢浩</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>王芳</t>
+          <t>胡金鑫</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-57897</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>依赖搜索引擎升级</t>
+          <t>因8.0需求变更，待重新评审</t>
         </is>
       </c>
     </row>
@@ -892,39 +920,43 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>9.8.0 (20260318)</t>
+          <t>8.1.1 (2024Q4)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>互动消息中心</t>
+          <t>社区v8.1需求（个人主页搜索/取消点赞/回复评论数）</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>统一的消息中心：整合点赞、评论、关注、@等通知类型；支持消息分组、一键已读、消息跳转至原文</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>3</v>
+          <t>个人主页搜索帖子、列表显示回复的评论数、取消点赞功能</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>张伟/李明/王强</t>
+          <t>王战胜/臧宝亮</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>王芳</t>
+          <t>周颖</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -932,10 +964,14 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58459</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>需与IM消息区分展示</t>
+          <t>需求拆分：搜索+评论数(1d)，取消点赞(1.5d)</t>
         </is>
       </c>
     </row>
@@ -945,50 +981,54 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>9.10.0 (20260506)</t>
+          <t>8.2.0 (2024Q4)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>帖子详情页改版</t>
+          <t>社区-草稿箱</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>帖子详情页UI重构：新增大图模式、相关推荐模块、评论区沉浸式体验、作者信息卡片增强</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>3</v>
+          <t>社区发帖草稿箱功能</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>张伟/李明</t>
+          <t>王战胜/臧宝亮</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>刘洋</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58521</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>设计稿评审中</t>
+          <t>长文草稿箱需要H5配合</t>
         </is>
       </c>
     </row>
@@ -998,47 +1038,55 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>9.10.0 (20260506)</t>
+          <t>8.2.0 (2024Q4)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>社区关注推荐优化</t>
+          <t>搜索用户、社区的优化</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>优化关注流推荐策略：新增'可能感兴趣的人'模块、好友关注动态提醒、创作者入驻引导</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>2</v>
+          <t>用户搜索和社区搜索功能优化</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>李明</t>
+          <t>王战胜/臧宝亮</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>刘洋</t>
+          <t>胡金鑫</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58824</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1047,39 +1095,43 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>10.6.0 (20260708)</t>
+          <t>8.3.0 (2024Q4)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>社区首页Feed流改版</t>
+          <t>24年社区首页改版</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>社区首页全面改版：Feed流样式升级（双列/单列切换）、视频自动播放、话题聚合卡片、直播入口</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>4</v>
+          <t>社区首页全面改版：关注Feed支持新闻评论/大V观点、热门feed、推荐&amp;热门顶部热门股票列表、推送数据给推荐系统</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>张伟/李明/王强</t>
+          <t>王战胜/臧宝亮</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>王芳</t>
+          <t>周颖</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1087,10 +1139,14 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58822</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>v10.6重点需求；含UI大改版</t>
+          <t>页面结构1d+帖子1d+新闻1d+大V观点3d+热门2d+推荐1d</t>
         </is>
       </c>
     </row>
@@ -1100,55 +1156,1093 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>secret (20260708)</t>
+          <t>8.3.0 (2024Q4)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>互动消息增加跳H5</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>互动消息支持跳转至H5页面</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>杨怀展/卢浩</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>胡金鑫</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-59006</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>8.3.0 (2024Q4)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>消息中心：点赞跳转优化</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>消息中心点赞消息的跳转体验优化</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>杨怀展/卢浩</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>胡金鑫</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-59373</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>8.4.0 (2024Q4)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>股吧帖子支持期货挂链</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>股吧帖子支持期货挂链功能</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>杨怀展/卢浩</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58476</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>8.4.0 (2024Q4)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>社区首页推荐feed曝光点击数据埋点增加recommend_info上报</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>社区首页推荐Feed流的曝光点击数据埋点增加recommend_info字段上报</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>王战胜/臧宝亮</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-59528</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>8.4.0 (2024Q4)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>股吧回复支持上传1张图片</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>股吧回复评论支持上传1张图片</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>杨怀展/卢浩</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-58454</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>8.5.0 (2024Q4)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>话题详情页分享帖子套用话题分享海报</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>话题详情页分享帖子时使用话题专属分享海报</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>王战胜</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>8.7.0 (2025.1)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>股吧评论列表页显示已公开自选图标icon</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>在股吧评论列表页显示用户已公开的自选股图标</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>可以上</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>王战胜/臧宝亮</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>周颖</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>http://jira.intra.sina.com.cn/browse/SINAFINANCE-60603</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>9.4.0 (20251203)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>评论区发图</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>支持用户在评论中发布图片，包含图片上传、预览、删除功能</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>张伟/李明</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>王芳</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>需兼容已有评论展示</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>9.4.0 (20251203)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>社区帖子推荐优化</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>优化社区首页Feed流推荐算法，新增'推荐'Tab页</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>李明/张伟</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>王芳</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>需A/B测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>9.4.0 (20251203)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>帖子点赞动效优化</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>优化帖子点赞按钮的交互动效</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>张伟</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>王芳</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>9.6.0 (20260114)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>创作者中心V2</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>创作者中心二期：数据看板、内容管理后台、收益提现模块</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>李明/张伟</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>刘洋</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>依赖社区数据中台V2接口</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>9.6.0 (20260114)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>帖子评论排序优化</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>评论支持按热度/时间排序切换；热评置顶；楼中楼优化</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>张伟</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>刘洋</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>9.6.0 (20260114)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Feed流性能优化</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>社区首页Feed流虚拟列表、图片懒加载、预加载</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>李明/张伟/王强</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>刘洋</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Harmony端适配</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>9.8.0 (20260318)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>社区搜索V3</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>帖子全文搜索、搜索联想词、分类筛选、热门搜索榜</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>李明/张伟</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>王芳</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>依赖搜索引擎升级</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>9.8.0 (20260318)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>互动消息中心</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>统一消息中心：点赞/评论/关注/@通知，消息分组、一键已读、跳转原文</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>张伟/李明/王强</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>王芳</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>需与IM消息区分</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>9.10.0 (20260506)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>帖子详情页改版</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>帖子详情页UI重构：大图模式、相关推荐、评论区沉浸式、作者信息卡片</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>张伟/李明</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>刘洋</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>设计稿评审中</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>9.10.0 (20260506)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>社区关注推荐优化</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>关注流推荐优化：可能感兴趣的人、好友动态提醒、创作者入驻引导</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>李明</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>刘洋</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>10.6.0 (20260708)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>社区首页Feed流改版</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>社区首页全面改版：双列/单列切换、视频自动播放、话题聚合、直播入口</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>张伟/李明/王强</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>王芳</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>v10.6重点需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>10.6.0 (20260708)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
           <t>评论系统升级</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>评论系统全面升级：支持表情回复、评论置顶/折叠（作者功能）、评论举报、敏感词过滤增强、评论审核后台</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>评论系统全面升级：表情回复、评论置顶/折叠、举报、敏感词过滤、审核后台</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>张伟/李明/王强</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>王芳</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>需配合审核中台；含后台管理</t>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>需配合审核中台</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M13"/>
+  <autoFilter ref="A1:M31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>